<commit_message>
Replace empty daily view with verified Kraken prices, candles and calculated pivots
</commit_message>
<xml_diff>
--- a/downloads/crypto-journal-2026-10-04.xlsx
+++ b/downloads/crypto-journal-2026-10-04.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="1" r:id="R6259f96e2288434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="1" r:id="R992059834cc9455b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="200" formatCode="dd.mm.yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0000"/>
     <x:numFmt numFmtId="202" formatCode="0.00%"/>
-    <x:numFmt numFmtId="203" formatCode="#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0.0"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -106,16 +106,16 @@
     <x:tableColumn id="1" name="Datum"/>
     <x:tableColumn id="2" name="Coin"/>
     <x:tableColumn id="3" name="Kurs (USDT)"/>
-    <x:tableColumn id="4" name="Trend (Heatmap)"/>
-    <x:tableColumn id="5" name="Support (Heatmap)"/>
-    <x:tableColumn id="6" name="Widerstand (Heatmap)"/>
+    <x:tableColumn id="4" name="Trend"/>
+    <x:tableColumn id="5" name="Support"/>
+    <x:tableColumn id="6" name="Widerstand"/>
     <x:tableColumn id="7" name="Long-Zone"/>
     <x:tableColumn id="8" name="Short-Zone"/>
     <x:tableColumn id="9" name="Breakout über"/>
     <x:tableColumn id="10" name="Breakdown unter"/>
     <x:tableColumn id="11" name="Ziele"/>
     <x:tableColumn id="12" name="Heatmap-Cluster"/>
-    <x:tableColumn id="13" name="Dominanz unterhalb"/>
+    <x:tableColumn id="13" name="Heatmap-Dominanz"/>
     <x:tableColumn id="14" name="Veränderung zum Vortag"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -340,7 +340,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Stand 2026-10-04; alle Kursmarken in USDT. Heatmap-Cluster wie in den Grafiken.</x:v>
+        <x:v>Stand 2026-10-04; Kraken Spot in USDT; technische Marken: berechnete Tagespivots.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="40" customHeight="1">
@@ -354,13 +354,13 @@
         <x:v>Kurs (USDT)</x:v>
       </x:c>
       <x:c r="D5" s="7" t="str">
-        <x:v>Trend (Heatmap)</x:v>
+        <x:v>Trend</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
-        <x:v>Support (Heatmap)</x:v>
+        <x:v>Support</x:v>
       </x:c>
       <x:c r="F5" s="7" t="str">
-        <x:v>Widerstand (Heatmap)</x:v>
+        <x:v>Widerstand</x:v>
       </x:c>
       <x:c r="G5" s="7" t="str">
         <x:v>Long-Zone</x:v>
@@ -381,7 +381,7 @@
         <x:v>Heatmap-Cluster</x:v>
       </x:c>
       <x:c r="M5" s="7" t="str">
-        <x:v>Dominanz unterhalb</x:v>
+        <x:v>Heatmap-Dominanz</x:v>
       </x:c>
       <x:c r="N5" s="7" t="str">
         <x:v>Veränderung zum Vortag</x:v>
@@ -394,41 +394,41 @@
       <x:c r="B6" s="4" t="str">
         <x:v>BTC</x:v>
       </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>Nicht verfügbar</x:v>
+      <x:c r="C6" s="11" t="n">
+        <x:v>85279.9</x:v>
       </x:c>
       <x:c r="D6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Über SMA20 (82.473,0); über Tagespivot 84.744,4</x:v>
       </x:c>
       <x:c r="E6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>S1 84.456,6 / S2 84.156,8</x:v>
       </x:c>
       <x:c r="F6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>R1 85.044,2 / R2 85.332,0</x:v>
       </x:c>
       <x:c r="G6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>84.456,6–84.744,4 (Pivot-Rücklauf; Bestätigung abwarten)</x:v>
       </x:c>
       <x:c r="H6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
-      </x:c>
-      <x:c r="I6" s="11" t="str">
-        <x:v>Nicht verfügbar</x:v>
-      </x:c>
-      <x:c r="J6" s="11" t="str">
-        <x:v>Nicht verfügbar</x:v>
+        <x:v>85.044,2–85.332,0 (nur bei Ablehnung)</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="n">
+        <x:v>85044.16666666667</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="n">
+        <x:v>84456.56666666667</x:v>
       </x:c>
       <x:c r="K6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Oberseite R1/R2: 85.044,2 / 85.332,0; Unterseite S1/S2: 84.456,6 / 84.156,8</x:v>
       </x:c>
       <x:c r="L6" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Keine aktuelle Liquidationsquelle; alte Heatmap: 03.10.2026</x:v>
       </x:c>
       <x:c r="M6" s="10" t="str">
         <x:v>Nicht verfügbar</x:v>
       </x:c>
-      <x:c r="N6" s="10" t="str">
-        <x:v>Nicht verfügbar</x:v>
+      <x:c r="N6" s="10" t="n">
+        <x:v>0.006177711863306845</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -438,46 +438,46 @@
       <x:c r="B7" s="4" t="str">
         <x:v>XRP</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>Nicht verfügbar</x:v>
+      <x:c r="C7" s="9" t="n">
+        <x:v>1.50113</x:v>
       </x:c>
       <x:c r="D7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Über SMA20 (1,4611); über Tagespivot 1,4875</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>S1 1,4794 / S2 1,4720</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>R1 1,4950 / R2 1,5030</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>1,4794–1,4875 (Pivot-Rücklauf; Bestätigung abwarten)</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
-      </x:c>
-      <x:c r="I7" s="9" t="str">
-        <x:v>Nicht verfügbar</x:v>
-      </x:c>
-      <x:c r="J7" s="9" t="str">
-        <x:v>Nicht verfügbar</x:v>
+        <x:v>1,4950–1,5030 (nur bei Ablehnung)</x:v>
+      </x:c>
+      <x:c r="I7" s="9" t="n">
+        <x:v>1.4949533333333334</x:v>
+      </x:c>
+      <x:c r="J7" s="9" t="n">
+        <x:v>1.4794233333333333</x:v>
       </x:c>
       <x:c r="K7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Oberseite R1/R2: 1,4950 / 1,5030; Unterseite S1/S2: 1,4794 / 1,4720</x:v>
       </x:c>
       <x:c r="L7" s="4" t="str">
-        <x:v>Nicht verfügbar · Quelle heute nicht verifiziert</x:v>
+        <x:v>Keine aktuelle Liquidationsquelle; alte Heatmap: 03.10.2026</x:v>
       </x:c>
       <x:c r="M7" s="10" t="str">
         <x:v>Nicht verfügbar</x:v>
       </x:c>
-      <x:c r="N7" s="10" t="str">
-        <x:v>Nicht verfügbar</x:v>
+      <x:c r="N7" s="10" t="n">
+        <x:v>0.009577036633510172</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="12" t="str">
-        <x:v>Erfasst: 04.10.2026, 11:35 Uhr Europe/Berlin. Binance-, Coinbase- und Kraken-APIs über den verfügbaren Abruf nicht zugänglich. Widersprüchliche USD-Indikationen wurden nicht als USDT-Kurse übernommen. Aktuelle Kurse, technische Marken und Heatmap-Daten nicht verfügbar. Charts: 03.10.2026. Vorhandener XRP-Eintrag vom 04.10. ohne Quellen/Zeitstempel unverändert als source-snapshot gesichert; nicht als verifizierte Tagesdaten übernommen.</x:v>
+        <x:v>Kraken Spot BTC/USDT und XRP/USDT. Abruf 04.10.2026, 11:45 Uhr Europe/Berlin; Börsenzeit bestätigt. Veränderung: aktueller letzter Handel gegen Kraken-Schlusskurs des 03.10.2026 (UTC), nicht gegen den älteren Journal-Screenshot. Trend: Kurs gegen SMA20 der abgeschlossenen UTC-Tage. Klassische Tagespivots: P=(Vortagshoch+Vortagstief+Vortagsschluss)/3; S1=2P-H, R1=2P-L, S2=P-(H-L), R2=P+(H-L). Zonen und Ziele sind daraus abgeleitete Szenarien; keine unabhängig bestätigten Chart-Signale. Aktuelle Liquidations-Heatmap fehlt; Grafikstand 03.10.2026 bleibt separat erhalten.</x:v>
       </x:c>
       <x:c r="B9" s="12"/>
       <x:c r="C9" s="12"/>
@@ -527,11 +527,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="12" t="str">
-        <x:v>https://api.binance.com/api/v3/ticker/24hr?symbol=BTCUSDT
-https://api.coinbase.com/v2/prices/BTC-USD/spot
-https://api.kraken.com/0/public/Ticker?pair=XBTUSDT,XRPUSDT
-https://ca.investing.com/crypto/bitcoin/historical-data
-https://ca.investing.com/crypto/xrp/historical-data</x:v>
+        <x:v>https://api.kraken.com/0/public/Ticker?pair=XBTUSDT,XRPUSDT
+https://api.kraken.com/0/public/OHLC?pair=XBTUSDT&amp;interval=1440
+https://api.kraken.com/0/public/OHLC?pair=XRPUSDT&amp;interval=1440
+https://api.kraken.com/0/public/Time</x:v>
       </x:c>
       <x:c r="B13" s="12"/>
       <x:c r="C13" s="12"/>
@@ -602,7 +601,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89aba7a75e844e7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26efdc40f1a44650"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>